<commit_message>
modified report document export function
</commit_message>
<xml_diff>
--- a/api/app/static/reports/payments/payment_1_202608.xlsx
+++ b/api/app/static/reports/payments/payment_1_202608.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -505,7 +505,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -541,7 +541,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -577,7 +577,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -613,7 +613,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -649,7 +649,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -685,7 +685,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -721,7 +721,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -757,7 +757,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -829,7 +829,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>unpaid</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="D13" t="n">

</xml_diff>